<commit_message>
updating org info and running tests
Will make release soon for OS 11.
</commit_message>
<xml_diff>
--- a/results/RESULTS5-4.xlsx
+++ b/results/RESULTS5-4.xlsx
@@ -1244,7 +1244,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.000000"/>
@@ -11027,7 +11027,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -11218,7 +11218,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet14"/>
   <dimension ref="A1:I97"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -11907,7 +11907,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet15"/>
   <dimension ref="A1:E134"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -12868,7 +12868,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet16"/>
   <dimension ref="A1:E124"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -13789,7 +13789,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet17"/>
   <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -14191,7 +14191,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet18"/>
   <dimension ref="A1:K169"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -14221,7 +14221,7 @@
         <v>38</v>
       </c>
       <c r="F2" s="377" t="str">
-        <v>EnergyPlus 25.1.0 , Bug Fix Edition</v>
+        <v>EnergyPlus 25.2.0 , Bug Fix Edition</v>
       </c>
       <c r="G2" s="378"/>
       <c r="H2" s="378"/>
@@ -14240,7 +14240,7 @@
       <c r="H3" s="349"/>
       <c r="I3" s="295"/>
       <c r="J3" s="360" t="str">
-        <v>05/28/25</v>
+        <v>11/14/25</v>
       </c>
       <c r="K3" s="108" t="s">
         <v>54</v>
@@ -14279,7 +14279,7 @@
       <c r="H5" s="349"/>
       <c r="I5" s="295"/>
       <c r="J5" s="360" t="str">
-        <v>06/18/2025</v>
+        <v>06/09/2026</v>
       </c>
       <c r="K5" s="109"/>
     </row>
@@ -14307,7 +14307,7 @@
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="377" t="str">
-        <v>National Renewable Energy Laboratory</v>
+        <v>National Laboratory of the Rockies</v>
       </c>
       <c r="G7" s="378"/>
       <c r="H7" s="378"/>
@@ -14328,7 +14328,7 @@
       <c r="H8" s="349"/>
       <c r="I8" s="349"/>
       <c r="J8" s="350" t="str">
-        <v>NREL</v>
+        <v>NLR</v>
       </c>
       <c r="K8" s="109"/>
     </row>
@@ -16382,7 +16382,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet2">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -16628,7 +16628,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet3">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -16942,7 +16942,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet5">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -17268,7 +17268,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:L519"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -25186,7 +25186,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A1:M62"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
@@ -26847,7 +26847,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:mv="urn:schemas-microsoft-com:mac:vml">
   <sheetPr codeName="Sheet13"/>
   <dimension ref="D1:J406"/>
   <sheetFormatPr defaultRowHeight="12.75"/>

</xml_diff>